<commit_message>
correcao planilha de instruções
</commit_message>
<xml_diff>
--- a/RCA 1802 - Instruções.xlsx
+++ b/RCA 1802 - Instruções.xlsx
@@ -6,7 +6,6 @@
     <sheet state="visible" name="Instruções" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="Modos de Endereçamento" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Tabela de Símbolos" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Guido" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -14,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="496">
   <si>
     <t>RCA 1802 — Conjunto de Instruções</t>
   </si>
@@ -1503,538 +1502,13 @@
   </si>
   <si>
     <t>Separador de micro-operações dentro de um mesmo ciclo de execute. Ex.: D → M(R(X)); R(X)-1 → R(X).</t>
-  </si>
-  <si>
-    <t>RCA 1802 — Guia de Preenchimento  |  Pessoa B</t>
-  </si>
-  <si>
-    <t>ALU Lógica  ·  Desvios Curtos  ·  Desvios Longos  ·  Controle e I/O  |  Prazo: 24/06 (D+2)</t>
-  </si>
-  <si>
-    <t>1.  O que você precisa fazer</t>
-  </si>
-  <si>
-    <t>Sua missão</t>
-  </si>
-  <si>
-    <t>Preencher todas as linhas das suas instruções na aba "Instruções - RCA 1802", seguindo exatamente o mesmo formato das linhas já preenchidas pela Pessoa A. Cada instrução deve ter as 14 colunas completas.</t>
-  </si>
-  <si>
-    <t>Onde preencher</t>
-  </si>
-  <si>
-    <t>Aba "Instruções - RCA 1802" → role até o fim das linhas da Pessoa A → comece uma nova linha de cabeçalho de categoria (igual às existentes) e adicione as suas instruções abaixo.</t>
-  </si>
-  <si>
-    <t>Como copiar o estilo</t>
-  </si>
-  <si>
-    <t>No Google Sheets: selecione uma linha de instrução já existente → Ctrl+C → clique na nova linha vazia → clique direito → "Colar especial &gt; Somente formatação". Depois edite apenas o conteúdo.</t>
-  </si>
-  <si>
-    <t>Deadline</t>
-  </si>
-  <si>
-    <t>Entrega para o grupo: 24/06 (D+2) até o fim do dia. Os Grupos 4 e 5 dependem desta tabela para começar. Não atrase.</t>
-  </si>
-  <si>
-    <t>2.  Suas instruções por categoria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ALU LÓGICA  —  6 instruções</t>
-  </si>
-  <si>
-    <t>F1  OR  [—]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Indireto Reg. X  |  Op: M(R(X)) OR D → D</t>
-  </si>
-  <si>
-    <t>F9  ORI  [imm]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Imediato  |  Op: M(R(P)) OR D → D; R(P) + 1 → R(P)</t>
-  </si>
-  <si>
-    <t>F2  AND  [—]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Indireto Reg. X  |  Op: M(R(X)) AND D → D</t>
-  </si>
-  <si>
-    <t>FA  ANI  [imm]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Imediato  |  Op: M(R(P)) AND D → D; R(P) + 1 → R(P)</t>
-  </si>
-  <si>
-    <t>F3  XOR  [—]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Indireto Reg. X  |  Op: M(R(X)) XOR D → D</t>
-  </si>
-  <si>
-    <t>FB  XRI  [imm]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Imediato  |  Op: M(R(P)) XOR D → D; R(P) + 1 → R(P)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  DESVIOS CURTOS  —  16 instruções (2 bytes, 2 ciclos de máq.)</t>
-  </si>
-  <si>
-    <t>30  BR  [addr]</t>
-  </si>
-  <si>
-    <t>Op: R(P).0 ← M(R(P)); sempre</t>
-  </si>
-  <si>
-    <t>31  BQ  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF Q=1, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>32  BZ  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF D=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>33  BDF  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF DF=1, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>34  B1  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF1=1, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>35  B2  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF2=1, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>36  B3  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF3=1, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>37  B4  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF4=1, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>38  SKP  [—]</t>
-  </si>
-  <si>
-    <t>Op: R(P) + 1 → R(P)  (também chamado NBR)</t>
-  </si>
-  <si>
-    <t>39  BNQ  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF Q=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>3A  BNZ  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF D≠0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>3B  BNF  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF DF=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>3C  BN1  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF1=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>3D  BN2  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF2=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>3E  BN3  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF3=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>3F  BN4  [addr]</t>
-  </si>
-  <si>
-    <t>Op: IF EF4=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  DESVIOS LONGOS E SKIPS LONGOS  —  16 instruções (3 bytes, 3 ciclos de máq. = 24 clocks)</t>
-  </si>
-  <si>
-    <t>C0  LBR  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: M(R(P)) → R(P).1; M(R(P)+1) → R(P).0; sempre</t>
-  </si>
-  <si>
-    <t>C1  LBQ  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: IF Q=1, M(R(P))→R(P).1, M(R(P)+1)→R(P).0; ELSE R(P)+2→R(P)</t>
-  </si>
-  <si>
-    <t>C2  LBZ  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: IF D=0, M(R(P))→R(P).1, M(R(P)+1)→R(P).0; ELSE R(P)+2→R(P)</t>
-  </si>
-  <si>
-    <t>C3  LBDF  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: IF DF=1, M(R(P))→R(P).1, M(R(P)+1)→R(P).0; ELSE R(P)+2→R(P)</t>
-  </si>
-  <si>
-    <t>C4  NOP  [—]</t>
-  </si>
-  <si>
-    <t>Op: Nenhuma operação  (3 ciclos de máquina)</t>
-  </si>
-  <si>
-    <t>C8  LSKP  [—]</t>
-  </si>
-  <si>
-    <t>Op: R(P) + 2 → R(P)  (também chamado NLBR)</t>
-  </si>
-  <si>
-    <t>C9  LBNQ  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: IF Q=0, M(R(P))→R(P).1, M(R(P)+1)→R(P).0; ELSE R(P)+2→R(P)</t>
-  </si>
-  <si>
-    <t>CA  LBNZ  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: IF D≠0, M(R(P))→R(P).1, M(R(P)+1)→R(P).0; ELSE R(P)+2→R(P)</t>
-  </si>
-  <si>
-    <t>CB  LBNF  [addr16]</t>
-  </si>
-  <si>
-    <t>Op: IF DF=0, M(R(P))→R(P).1, M(R(P)+1)→R(P).0; ELSE R(P)+2→R(P)</t>
-  </si>
-  <si>
-    <t>C5  LSNQ  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF Q=0, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t>C6  LSNZ  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF D≠0, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t>C7  LSNF  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF DF=0, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t>CC  LSIE  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF IE=1, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t>CD  LSQ  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF Q=1, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t>CE  LSZ  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF D=0, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t>CF  LSDF  [—]</t>
-  </si>
-  <si>
-    <t>Op: IF DF=1, R(P)+2→R(P); ELSE continua</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  CONTROLE E I/O  —  20 instruções</t>
-  </si>
-  <si>
-    <t>61–67  OUT 1–7  [p (1-7)]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Ind.Reg.X+AutoInc  |  Op: M(R(X)) → BUS; R(X)+1 → R(X); N=p  (7 opcodes)</t>
-  </si>
-  <si>
-    <t>69–6F  IN 1–7  [p (1-7)]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Ind.Reg.X  |  Op: BUS → M(R(X)); BUS → D; N=p+8  (7 opcodes; 68h não existe)</t>
-  </si>
-  <si>
-    <t>7A  REQ  [—]</t>
-  </si>
-  <si>
-    <t>Flags: Q  |  Modo: —  |  Op: 0 → Q</t>
-  </si>
-  <si>
-    <t>7B  SEQ  [—]</t>
-  </si>
-  <si>
-    <t>Flags: Q  |  Modo: —  |  Op: 1 → Q</t>
-  </si>
-  <si>
-    <t>78  SAV  [—]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Ind.Reg.X  |  Op: T → M(R(X))</t>
-  </si>
-  <si>
-    <t>79  MARK  [—]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: Ind.Reg.2  |  Op: (X,P) → T; T → M(R(2)); P → X; R(2)-1 → R(2)</t>
-  </si>
-  <si>
-    <t>70  RET  [—]</t>
-  </si>
-  <si>
-    <t>Flags: IE,X,P  |  Modo: Ind.Reg.X  |  Op: M(R(X)) → (X,P); R(X)+1 → R(X); 1 → IE</t>
-  </si>
-  <si>
-    <t>71  DIS  [—]</t>
-  </si>
-  <si>
-    <t>Flags: IE,X,P  |  Modo: Ind.Reg.X  |  Op: M(R(X)) → (X,P); R(X)+1 → R(X); 0 → IE</t>
-  </si>
-  <si>
-    <t>00  IDL  [—]</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: —  |  Op: WAIT FOR DMA OR INTERRUPT; M(R(0)) → BUS  (controle)</t>
-  </si>
-  <si>
-    <t>Flags: nenhuma  |  Modo: —  |  Op: Nenhuma operação  (já listado em Desvios Longos)</t>
-  </si>
-  <si>
-    <t>3.  O que preencher em cada coluna</t>
-  </si>
-  <si>
-    <t>Nome do bloco: ALU LÓGICA / DESVIOS CURTOS / DESVIOS LONGOS / CONTROLE E I/O</t>
-  </si>
-  <si>
-    <t>Opcode em hexadecimal. Para instruções com nibble variável: 0N, 4N, etc. Para ranges fixos: 61–67.</t>
-  </si>
-  <si>
-    <t>Hex convertido em binário, separando nibbles com " | ". Ex.: F1 → 1111 | 0001. Para variável: 1111 | NNNN.</t>
-  </si>
-  <si>
-    <t>Os 4 bits superiores do opcode (classe da instrução). Ex.: OR (F1) → I = 1111.</t>
-  </si>
-  <si>
-    <t>Os 4 bits inferiores. Para instruções fixas, é constante. Para instruções de registrador, é NNNN (0–F).</t>
-  </si>
-  <si>
-    <t>Nome exato da Tabela 1 do datasheet Intersil. Se houver nome alternativo, coloque entre parênteses: SKP (≡ NBR).</t>
-  </si>
-  <si>
-    <t>"—" para nenhum, "n" para registrador, "imm" para imediato, "addr" para endereço curto (1 byte), "addr16" para endereço longo (2 bytes).</t>
-  </si>
-  <si>
-    <t>1 byte (sem operando), 2 bytes (com imm ou addr), 3 bytes (com addr16). Todos os desvios longos e skips longos = 3 bytes.</t>
-  </si>
-  <si>
-    <t>2 para quase tudo. EXCEÇÃO: todos os desvios longos, skips longos e NOP = 3.</t>
-  </si>
-  <si>
-    <t>Sempre Ciclos Máq. × 8. Portanto: 16 ou 24.</t>
-  </si>
-  <si>
-    <t>"nenhuma" para lógicas e desvios. "DF" para aritméticas e shifts. "Q" para SEQ/REQ. "IE, X, P" para RET e DIS.</t>
-  </si>
-  <si>
-    <t>Use exatamente estes nomes: Indireto Reg. X / Imediato / Página / Absoluto / Reg. direto / Indireto Reg. X + AutoInc / — (para instruções sem acesso a memória).</t>
-  </si>
-  <si>
-    <t>Copie da Tabela 1 do datasheet (págs. 3-23 a 3-26). Use seta → para atribuição, ponto-e-vírgula ; para separar micro-operações, e IF/ELSE para condições. Não invente notação própria.</t>
-  </si>
-  <si>
-    <t>Referência à figura da Tabela 2 do datasheet (ex: "Ver Fig. 8"), mnemônicos alternativos, comportamentos especiais ou armadilhas.</t>
-  </si>
-  <si>
-    <t>4.  Armadilhas específicas das suas instruções</t>
-  </si>
-  <si>
-    <t>⚠  ALU Lógica — DF não é afetado</t>
-  </si>
-  <si>
-    <t>OR, AND e XOR NÃO alteram o flag DF. A coluna "Flags Afetadas" deve conter "nenhuma" para todas as 6 instruções lógicas. Erro muito comum.</t>
-  </si>
-  <si>
-    <t>⚠  Desvios Curtos — o que acontece quando a condição NÃO é satisfeita</t>
-  </si>
-  <si>
-    <t>Quando a condição é FALSA, o byte de endereço é pulado: R(P)+1 → R(P). A instrução NÃO faz nada além de avançar o PC. Inclua o ELSE na notação formal: "IF cond, M(R(P))→R(P).0; ELSE R(P)+1→R(P)".</t>
-  </si>
-  <si>
-    <t>⚠  Desvios Curtos — endereçamento por página</t>
-  </si>
-  <si>
-    <t>Os desvios curtos carregam o byte de endereço SOMENTE em R(P).0 (byte baixo). O byte alto de R(P) não muda. Isso restringe o salto à mesma página de 256 bytes onde está o byte de endereço. Modo = "Página" (não "Absoluto").</t>
-  </si>
-  <si>
-    <t>⚠  Desvios Longos — ciclos de máquina = 3 (não 2)</t>
-  </si>
-  <si>
-    <t>TODOS os desvios longos (LBR, LBQ, LBZ, LBDF, LBNQ, LBNZ, LBNF), os skips longos (LSKP, LSNQ, LSNZ, LSNF, LSQ, LSDF, LSZ, LSIE) e o NOP consomem 3 ciclos de máquina = 24 ciclos de clock. Coluna "Ciclos Máq." = 3, "Ciclos Clock" = 24.</t>
-  </si>
-  <si>
-    <t>⚠  Desvios Longos — quando condição NÃO satisfeita, pula 2 bytes</t>
-  </si>
-  <si>
-    <t>Quando a condição é FALSA em um desvio longo, R(P)+2 → R(P) (pula os dois bytes de endereço). Diferente dos curtos que pulam apenas 1 byte.</t>
-  </si>
-  <si>
-    <t>⚠  SKP (38) e LSKP (C8) têm mnemônicos alternativos</t>
-  </si>
-  <si>
-    <t>SKP (38) também é chamado NBR ("No Branch"). LSKP (C8) também é chamado NLBR ("No Long Branch"). Registre os dois na coluna Mnemônico: "SKP (≡ NBR)".</t>
-  </si>
-  <si>
-    <t>⚠  Opcode 68h não existe</t>
-  </si>
-  <si>
-    <t>O mapa de opcodes pula de 67h (OUT 7) direto para 69h (IN 1). O opcode 68h não está definido. Mencione isso nas Observações do bloco IN/OUT.</t>
-  </si>
-  <si>
-    <t>⚠  OUT — MRD ativo (lê da memória para enviar ao barramento)</t>
-  </si>
-  <si>
-    <t>A instrução OUT FAZ uma leitura de memória (MRD=0) para colocar M(R(X)) no barramento de saída. R(X) é incrementado após. Modo = "Indireto Reg. X + AutoInc". Ver Fig. 11 da Tabela 2.</t>
-  </si>
-  <si>
-    <t>⚠  IN — escreve simultaneamente em M(R(X)) E em D</t>
-  </si>
-  <si>
-    <t>A instrução IN copia o BUS de entrada para DOIS destinos ao mesmo tempo: M(R(X)) e D. Notação: "BUS → M(R(X)); BUS → D". R(X) NÃO é incrementado. Ver Fig. 10.</t>
-  </si>
-  <si>
-    <t>⚠  RET e DIS — operação exata da Tabela 1</t>
-  </si>
-  <si>
-    <t>Use a notação exata: "M(R(X)) → (X,P); R(X)+1 → R(X); 1/0 → IE". O conteúdo de M(R(X)) vai para AMBOS X e P simultaneamente (X recebe o nibble alto, P o nibble baixo). Ver Fig. 8.</t>
-  </si>
-  <si>
-    <t>⚠  MARK — operação complexa</t>
-  </si>
-  <si>
-    <t>Sequência: (1) salva X:P no temporário T; (2) copia T para M(R(2)); (3) P → X (X passa a apontar para o mesmo registrador que era o PC); (4) R(2) é decrementado. Notação: "(X,P) → T; T → M(R(2)); P → X; R(2)-1 → R(2)".</t>
-  </si>
-  <si>
-    <t>5.  Regras de notação formal (coluna "Operação")</t>
-  </si>
-  <si>
-    <t>Atribuição / transferência.  Ex.: M(R(P)) → D</t>
-  </si>
-  <si>
-    <t>Separa micro-operações dentro do mesmo ciclo Execute.  Ex.: M(R(X)) → D; R(X)+1 → R(X)</t>
-  </si>
-  <si>
-    <t>IF/ELSE</t>
-  </si>
-  <si>
-    <t>Para desvios condicionais.  Ex.: IF D=0, M(R(P)) → R(P).0; ELSE R(P)+1 → R(P)</t>
-  </si>
-  <si>
-    <t>R(P).0</t>
-  </si>
-  <si>
-    <t>Byte baixo (bits 7–0) do registrador PC. Usado nos desvios curtos.</t>
-  </si>
-  <si>
-    <t>R(P).1</t>
-  </si>
-  <si>
-    <t>Byte alto (bits 15–8) do registrador PC. Usado nos desvios longos.</t>
-  </si>
-  <si>
-    <t>Barramento externo de dados/endereços. Usado em OUT, IN e IDL.</t>
-  </si>
-  <si>
-    <t>(X,P)</t>
-  </si>
-  <si>
-    <t>Leitura ou escrita simultânea dos dois campos X e P num único byte: X=nibble alto, P=nibble baixo.</t>
-  </si>
-  <si>
-    <t>Complemento de DF — borrow de entrada nas instruções SDB, SDBI, SMB, SMBI.</t>
-  </si>
-  <si>
-    <t>6.  Onde consultar</t>
-  </si>
-  <si>
-    <t>Tabela 1 do datasheet</t>
-  </si>
-  <si>
-    <t>cosmacelf.com/publications/data-sheets/cdp1802.pdf  →  págs. 3-23 a 3-26
-Fonte primária para mnemônicos, opcodes e notação formal das operações.</t>
-  </si>
-  <si>
-    <t>Tabela 2 do datasheet</t>
-  </si>
-  <si>
-    <t>Mesma URL  →  págs. 3-27 a 3-29
-Mostra estado do barramento (MRD, MWR, DATA, ADDR) por instrução durante o Execute.
-Referência obrigatória para a coluna Observações (qual Fig. citar).</t>
-  </si>
-  <si>
-    <t>Nota 4 da Tabela 1</t>
-  </si>
-  <si>
-    <t>Confirma que desvios longos, skips longos e NOP requerem 3 ciclos de máquina.</t>
-  </si>
-  <si>
-    <t>Nota 1 da Tabela 1</t>
-  </si>
-  <si>
-    <t>Confirma que SOMENTE aritméticas e shifts alteram DF. Lógicas (OR, AND, XOR) NÃO alteram DF.</t>
-  </si>
-  <si>
-    <t>Exemplo de referência</t>
-  </si>
-  <si>
-    <t>Veja as linhas da Pessoa A na aba "Instruções - RCA 1802" como modelo de formato, estilo e nível de detalhe esperado.</t>
-  </si>
-  <si>
-    <t>Dúvidas de notação ou conteúdo: consulte a Pessoa A ou o datasheet antes de preencher.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="44">
+  <fonts count="32">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -2207,76 +1681,8 @@
       <color rgb="FF5F5E5A"/>
       <name val="Courier New"/>
     </font>
-    <font>
-      <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FFD5E8F4"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
-      <color rgb="FF2C2C2A"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
-      <color rgb="FF993C1D"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
-      <color rgb="FF2C2C2A"/>
-      <name val="Courier New"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF0F6E56"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF993C1D"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF1A237E"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF1B4F8A"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="8.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2439,44 +1845,8 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF993C1D"/>
-        <bgColor rgb="FF993C1D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFAECE7"/>
-        <bgColor rgb="FFFAECE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0F6E56"/>
-        <bgColor rgb="FF0F6E56"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE1F5EE"/>
-        <bgColor rgb="FFE1F5EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEBF5FB"/>
-        <bgColor rgb="FFEBF5FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD5E8F4"/>
-        <bgColor rgb="FFD5E8F4"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="25">
+  <borders count="17">
     <border/>
     <border>
       <left/>
@@ -2650,123 +2020,11 @@
         <color rgb="FFB7B7B7"/>
       </bottom>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF993C1D"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFEDE7F6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFE1F5EE"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFFCE4D6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFFAECE7"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF0F6E56"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFEBF5FB"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFD5E8F4"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="302">
+  <cellXfs count="279">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3592,71 +2850,6 @@
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="27" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="32" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="33" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="19" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="27" fontId="19" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="3" fontId="35" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="27" fontId="36" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="17" fillId="28" fontId="35" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="29" fontId="37" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="12" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="18" fillId="13" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="27" fontId="38" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="30" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="19" fillId="31" fontId="39" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="20" fillId="7" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="28" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="21" fillId="29" fontId="40" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="22" fillId="30" fontId="35" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="28" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="23" fillId="32" fontId="41" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="24" fillId="33" fontId="42" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="43" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3676,10 +2869,6 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -10775,1858 +9964,4 @@
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="3.0"/>
-    <col customWidth="1" min="2" max="2" width="28.0"/>
-    <col customWidth="1" min="3" max="3" width="75.0"/>
-    <col customWidth="1" min="4" max="4" width="3.0"/>
-    <col customWidth="1" min="5" max="26" width="8.71"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30.0" customHeight="1">
-      <c r="A1" s="279" t="s">
-        <v>496</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
-    </row>
-    <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="280" t="s">
-        <v>497</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" ht="7.5" customHeight="1">
-      <c r="A3" s="281"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="282" t="s">
-        <v>498</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="3"/>
-    </row>
-    <row r="5" ht="6.0" customHeight="1">
-      <c r="A5" s="283"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" ht="43.5" customHeight="1">
-      <c r="B6" s="284" t="s">
-        <v>499</v>
-      </c>
-      <c r="C6" s="285" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="7" ht="37.5" customHeight="1">
-      <c r="B7" s="284" t="s">
-        <v>501</v>
-      </c>
-      <c r="C7" s="285" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="8" ht="37.5" customHeight="1">
-      <c r="B8" s="284" t="s">
-        <v>503</v>
-      </c>
-      <c r="C8" s="285" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="9" ht="31.5" customHeight="1">
-      <c r="B9" s="286" t="s">
-        <v>505</v>
-      </c>
-      <c r="C9" s="287" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="10" ht="6.0" customHeight="1">
-      <c r="A10" s="283"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="282" t="s">
-        <v>507</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" ht="6.0" customHeight="1">
-      <c r="A12" s="283"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" ht="18.0" customHeight="1">
-      <c r="A13" s="288" t="s">
-        <v>508</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="B14" s="289" t="s">
-        <v>509</v>
-      </c>
-      <c r="C14" s="290" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="B15" s="289" t="s">
-        <v>511</v>
-      </c>
-      <c r="C15" s="290" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="B16" s="289" t="s">
-        <v>513</v>
-      </c>
-      <c r="C16" s="290" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="B17" s="289" t="s">
-        <v>515</v>
-      </c>
-      <c r="C17" s="290" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="B18" s="289" t="s">
-        <v>517</v>
-      </c>
-      <c r="C18" s="290" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="B19" s="289" t="s">
-        <v>519</v>
-      </c>
-      <c r="C19" s="290" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="20" ht="6.0" customHeight="1">
-      <c r="A20" s="283"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="3"/>
-    </row>
-    <row r="21" ht="18.0" customHeight="1">
-      <c r="A21" s="291" t="s">
-        <v>521</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="3"/>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="B22" s="292" t="s">
-        <v>522</v>
-      </c>
-      <c r="C22" s="290" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="B23" s="292" t="s">
-        <v>524</v>
-      </c>
-      <c r="C23" s="290" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="B24" s="292" t="s">
-        <v>526</v>
-      </c>
-      <c r="C24" s="290" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="B25" s="292" t="s">
-        <v>528</v>
-      </c>
-      <c r="C25" s="290" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="B26" s="292" t="s">
-        <v>530</v>
-      </c>
-      <c r="C26" s="290" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="B27" s="292" t="s">
-        <v>532</v>
-      </c>
-      <c r="C27" s="290" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="28" ht="21.75" customHeight="1">
-      <c r="B28" s="292" t="s">
-        <v>534</v>
-      </c>
-      <c r="C28" s="290" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="29" ht="21.75" customHeight="1">
-      <c r="B29" s="292" t="s">
-        <v>536</v>
-      </c>
-      <c r="C29" s="290" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="30" ht="21.75" customHeight="1">
-      <c r="B30" s="292" t="s">
-        <v>538</v>
-      </c>
-      <c r="C30" s="290" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="31" ht="21.75" customHeight="1">
-      <c r="B31" s="292" t="s">
-        <v>540</v>
-      </c>
-      <c r="C31" s="290" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="32" ht="21.75" customHeight="1">
-      <c r="B32" s="292" t="s">
-        <v>542</v>
-      </c>
-      <c r="C32" s="290" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="33" ht="21.75" customHeight="1">
-      <c r="B33" s="292" t="s">
-        <v>544</v>
-      </c>
-      <c r="C33" s="290" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="34" ht="21.75" customHeight="1">
-      <c r="B34" s="292" t="s">
-        <v>546</v>
-      </c>
-      <c r="C34" s="290" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="35" ht="21.75" customHeight="1">
-      <c r="B35" s="292" t="s">
-        <v>548</v>
-      </c>
-      <c r="C35" s="290" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="36" ht="21.75" customHeight="1">
-      <c r="B36" s="292" t="s">
-        <v>550</v>
-      </c>
-      <c r="C36" s="290" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="37" ht="21.75" customHeight="1">
-      <c r="B37" s="292" t="s">
-        <v>552</v>
-      </c>
-      <c r="C37" s="290" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="38" ht="6.0" customHeight="1">
-      <c r="A38" s="283"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="3"/>
-    </row>
-    <row r="39" ht="18.0" customHeight="1">
-      <c r="A39" s="293" t="s">
-        <v>554</v>
-      </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="3"/>
-    </row>
-    <row r="40" ht="21.75" customHeight="1">
-      <c r="B40" s="294" t="s">
-        <v>555</v>
-      </c>
-      <c r="C40" s="290" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="41" ht="21.75" customHeight="1">
-      <c r="B41" s="294" t="s">
-        <v>557</v>
-      </c>
-      <c r="C41" s="290" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="42" ht="21.75" customHeight="1">
-      <c r="B42" s="294" t="s">
-        <v>559</v>
-      </c>
-      <c r="C42" s="290" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="43" ht="21.75" customHeight="1">
-      <c r="B43" s="294" t="s">
-        <v>561</v>
-      </c>
-      <c r="C43" s="290" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="44" ht="21.75" customHeight="1">
-      <c r="B44" s="294" t="s">
-        <v>563</v>
-      </c>
-      <c r="C44" s="290" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="45" ht="21.75" customHeight="1">
-      <c r="B45" s="294" t="s">
-        <v>565</v>
-      </c>
-      <c r="C45" s="290" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="46" ht="21.75" customHeight="1">
-      <c r="B46" s="294" t="s">
-        <v>567</v>
-      </c>
-      <c r="C46" s="290" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="47" ht="21.75" customHeight="1">
-      <c r="B47" s="294" t="s">
-        <v>569</v>
-      </c>
-      <c r="C47" s="290" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="48" ht="21.75" customHeight="1">
-      <c r="B48" s="294" t="s">
-        <v>571</v>
-      </c>
-      <c r="C48" s="290" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="49" ht="21.75" customHeight="1">
-      <c r="B49" s="294" t="s">
-        <v>573</v>
-      </c>
-      <c r="C49" s="290" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="50" ht="21.75" customHeight="1">
-      <c r="B50" s="294" t="s">
-        <v>575</v>
-      </c>
-      <c r="C50" s="290" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="51" ht="21.75" customHeight="1">
-      <c r="B51" s="294" t="s">
-        <v>577</v>
-      </c>
-      <c r="C51" s="290" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="52" ht="21.75" customHeight="1">
-      <c r="B52" s="294" t="s">
-        <v>579</v>
-      </c>
-      <c r="C52" s="290" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="53" ht="21.75" customHeight="1">
-      <c r="B53" s="294" t="s">
-        <v>581</v>
-      </c>
-      <c r="C53" s="290" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="54" ht="21.75" customHeight="1">
-      <c r="B54" s="294" t="s">
-        <v>583</v>
-      </c>
-      <c r="C54" s="290" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="55" ht="21.75" customHeight="1">
-      <c r="B55" s="294" t="s">
-        <v>585</v>
-      </c>
-      <c r="C55" s="290" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="56" ht="6.0" customHeight="1">
-      <c r="A56" s="283"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="3"/>
-    </row>
-    <row r="57" ht="18.0" customHeight="1">
-      <c r="A57" s="295" t="s">
-        <v>587</v>
-      </c>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="3"/>
-    </row>
-    <row r="58" ht="21.75" customHeight="1">
-      <c r="B58" s="296" t="s">
-        <v>588</v>
-      </c>
-      <c r="C58" s="290" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="59" ht="21.75" customHeight="1">
-      <c r="B59" s="296" t="s">
-        <v>590</v>
-      </c>
-      <c r="C59" s="290" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="60" ht="21.75" customHeight="1">
-      <c r="B60" s="296" t="s">
-        <v>592</v>
-      </c>
-      <c r="C60" s="290" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="61" ht="21.75" customHeight="1">
-      <c r="B61" s="296" t="s">
-        <v>594</v>
-      </c>
-      <c r="C61" s="290" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="62" ht="21.75" customHeight="1">
-      <c r="B62" s="296" t="s">
-        <v>596</v>
-      </c>
-      <c r="C62" s="290" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="63" ht="21.75" customHeight="1">
-      <c r="B63" s="296" t="s">
-        <v>598</v>
-      </c>
-      <c r="C63" s="290" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="64" ht="21.75" customHeight="1">
-      <c r="B64" s="296" t="s">
-        <v>600</v>
-      </c>
-      <c r="C64" s="290" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="65" ht="21.75" customHeight="1">
-      <c r="B65" s="296" t="s">
-        <v>602</v>
-      </c>
-      <c r="C65" s="290" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="66" ht="21.75" customHeight="1">
-      <c r="B66" s="296" t="s">
-        <v>604</v>
-      </c>
-      <c r="C66" s="290" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="67" ht="21.75" customHeight="1">
-      <c r="B67" s="296" t="s">
-        <v>563</v>
-      </c>
-      <c r="C67" s="290" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="68" ht="6.0" customHeight="1">
-      <c r="A68" s="283"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="3"/>
-    </row>
-    <row r="69" ht="21.75" customHeight="1">
-      <c r="A69" s="282" t="s">
-        <v>607</v>
-      </c>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="3"/>
-    </row>
-    <row r="70" ht="6.0" customHeight="1">
-      <c r="A70" s="283"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="3"/>
-    </row>
-    <row r="71" ht="36.0" customHeight="1">
-      <c r="B71" s="284" t="s">
-        <v>1</v>
-      </c>
-      <c r="C71" s="285" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="72" ht="36.0" customHeight="1">
-      <c r="B72" s="284" t="s">
-        <v>2</v>
-      </c>
-      <c r="C72" s="285" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="73" ht="36.0" customHeight="1">
-      <c r="B73" s="284" t="s">
-        <v>3</v>
-      </c>
-      <c r="C73" s="285" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="74" ht="36.0" customHeight="1">
-      <c r="B74" s="284" t="s">
-        <v>4</v>
-      </c>
-      <c r="C74" s="285" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="75" ht="36.0" customHeight="1">
-      <c r="B75" s="284" t="s">
-        <v>5</v>
-      </c>
-      <c r="C75" s="285" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="76" ht="36.0" customHeight="1">
-      <c r="B76" s="284" t="s">
-        <v>6</v>
-      </c>
-      <c r="C76" s="285" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="77" ht="36.0" customHeight="1">
-      <c r="B77" s="284" t="s">
-        <v>7</v>
-      </c>
-      <c r="C77" s="285" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="78" ht="36.0" customHeight="1">
-      <c r="B78" s="284" t="s">
-        <v>8</v>
-      </c>
-      <c r="C78" s="285" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="79" ht="36.0" customHeight="1">
-      <c r="B79" s="286" t="s">
-        <v>9</v>
-      </c>
-      <c r="C79" s="285" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="80" ht="36.0" customHeight="1">
-      <c r="B80" s="284" t="s">
-        <v>10</v>
-      </c>
-      <c r="C80" s="285" t="s">
-        <v>617</v>
-      </c>
-    </row>
-    <row r="81" ht="36.0" customHeight="1">
-      <c r="B81" s="286" t="s">
-        <v>11</v>
-      </c>
-      <c r="C81" s="285" t="s">
-        <v>618</v>
-      </c>
-    </row>
-    <row r="82" ht="36.0" customHeight="1">
-      <c r="B82" s="284" t="s">
-        <v>12</v>
-      </c>
-      <c r="C82" s="285" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="83" ht="36.0" customHeight="1">
-      <c r="B83" s="297" t="s">
-        <v>13</v>
-      </c>
-      <c r="C83" s="285" t="s">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="84" ht="36.0" customHeight="1">
-      <c r="B84" s="284" t="s">
-        <v>14</v>
-      </c>
-      <c r="C84" s="285" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="85" ht="6.0" customHeight="1">
-      <c r="A85" s="283"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="3"/>
-    </row>
-    <row r="86" ht="21.75" customHeight="1">
-      <c r="A86" s="298" t="s">
-        <v>622</v>
-      </c>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="3"/>
-    </row>
-    <row r="87" ht="6.0" customHeight="1">
-      <c r="A87" s="283"/>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="3"/>
-    </row>
-    <row r="88" ht="43.5" customHeight="1">
-      <c r="B88" s="296" t="s">
-        <v>623</v>
-      </c>
-      <c r="C88" s="285" t="s">
-        <v>624</v>
-      </c>
-    </row>
-    <row r="89" ht="43.5" customHeight="1">
-      <c r="B89" s="292" t="s">
-        <v>625</v>
-      </c>
-      <c r="C89" s="285" t="s">
-        <v>626</v>
-      </c>
-    </row>
-    <row r="90" ht="43.5" customHeight="1">
-      <c r="B90" s="292" t="s">
-        <v>627</v>
-      </c>
-      <c r="C90" s="285" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="91" ht="43.5" customHeight="1">
-      <c r="B91" s="294" t="s">
-        <v>629</v>
-      </c>
-      <c r="C91" s="285" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="92" ht="43.5" customHeight="1">
-      <c r="B92" s="294" t="s">
-        <v>631</v>
-      </c>
-      <c r="C92" s="285" t="s">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="93" ht="43.5" customHeight="1">
-      <c r="B93" s="289" t="s">
-        <v>633</v>
-      </c>
-      <c r="C93" s="285" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="94" ht="43.5" customHeight="1">
-      <c r="B94" s="296" t="s">
-        <v>635</v>
-      </c>
-      <c r="C94" s="285" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="95" ht="43.5" customHeight="1">
-      <c r="B95" s="296" t="s">
-        <v>637</v>
-      </c>
-      <c r="C95" s="285" t="s">
-        <v>638</v>
-      </c>
-    </row>
-    <row r="96" ht="43.5" customHeight="1">
-      <c r="B96" s="296" t="s">
-        <v>639</v>
-      </c>
-      <c r="C96" s="285" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="97" ht="43.5" customHeight="1">
-      <c r="B97" s="296" t="s">
-        <v>641</v>
-      </c>
-      <c r="C97" s="285" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="98" ht="43.5" customHeight="1">
-      <c r="B98" s="296" t="s">
-        <v>643</v>
-      </c>
-      <c r="C98" s="285" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="99" ht="6.0" customHeight="1">
-      <c r="A99" s="283"/>
-      <c r="B99" s="2"/>
-      <c r="C99" s="2"/>
-      <c r="D99" s="3"/>
-    </row>
-    <row r="100" ht="21.75" customHeight="1">
-      <c r="A100" s="282" t="s">
-        <v>645</v>
-      </c>
-      <c r="B100" s="2"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="3"/>
-    </row>
-    <row r="101" ht="6.0" customHeight="1">
-      <c r="A101" s="283"/>
-      <c r="B101" s="2"/>
-      <c r="C101" s="2"/>
-      <c r="D101" s="3"/>
-    </row>
-    <row r="102" ht="25.5" customHeight="1">
-      <c r="B102" s="299" t="s">
-        <v>490</v>
-      </c>
-      <c r="C102" s="290" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="103" ht="25.5" customHeight="1">
-      <c r="B103" s="299" t="s">
-        <v>493</v>
-      </c>
-      <c r="C103" s="290" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="104" ht="25.5" customHeight="1">
-      <c r="B104" s="299" t="s">
-        <v>648</v>
-      </c>
-      <c r="C104" s="290" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="105" ht="25.5" customHeight="1">
-      <c r="B105" s="299" t="s">
-        <v>650</v>
-      </c>
-      <c r="C105" s="290" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="106" ht="25.5" customHeight="1">
-      <c r="B106" s="299" t="s">
-        <v>652</v>
-      </c>
-      <c r="C106" s="290" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="107" ht="25.5" customHeight="1">
-      <c r="B107" s="299" t="s">
-        <v>487</v>
-      </c>
-      <c r="C107" s="290" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="108" ht="25.5" customHeight="1">
-      <c r="B108" s="299" t="s">
-        <v>655</v>
-      </c>
-      <c r="C108" s="290" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="109" ht="25.5" customHeight="1">
-      <c r="B109" s="299" t="s">
-        <v>479</v>
-      </c>
-      <c r="C109" s="290" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="110" ht="6.0" customHeight="1">
-      <c r="A110" s="283"/>
-      <c r="B110" s="2"/>
-      <c r="C110" s="2"/>
-      <c r="D110" s="3"/>
-    </row>
-    <row r="111" ht="21.75" customHeight="1">
-      <c r="A111" s="282" t="s">
-        <v>658</v>
-      </c>
-      <c r="B111" s="2"/>
-      <c r="C111" s="2"/>
-      <c r="D111" s="3"/>
-    </row>
-    <row r="112" ht="6.0" customHeight="1">
-      <c r="A112" s="283"/>
-      <c r="B112" s="2"/>
-      <c r="C112" s="2"/>
-      <c r="D112" s="3"/>
-    </row>
-    <row r="113" ht="49.5" customHeight="1">
-      <c r="B113" s="300" t="s">
-        <v>659</v>
-      </c>
-      <c r="C113" s="285" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="114" ht="49.5" customHeight="1">
-      <c r="B114" s="300" t="s">
-        <v>661</v>
-      </c>
-      <c r="C114" s="285" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="115" ht="49.5" customHeight="1">
-      <c r="B115" s="300" t="s">
-        <v>663</v>
-      </c>
-      <c r="C115" s="285" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="116" ht="49.5" customHeight="1">
-      <c r="B116" s="300" t="s">
-        <v>665</v>
-      </c>
-      <c r="C116" s="285" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="117" ht="49.5" customHeight="1">
-      <c r="B117" s="300" t="s">
-        <v>667</v>
-      </c>
-      <c r="C117" s="285" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="118" ht="6.0" customHeight="1">
-      <c r="A118" s="283"/>
-      <c r="B118" s="2"/>
-      <c r="C118" s="2"/>
-      <c r="D118" s="3"/>
-    </row>
-    <row r="119" ht="18.0" customHeight="1">
-      <c r="A119" s="301" t="s">
-        <v>669</v>
-      </c>
-      <c r="B119" s="2"/>
-      <c r="C119" s="2"/>
-      <c r="D119" s="3"/>
-    </row>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="A99:D99"/>
-    <mergeCell ref="A100:D100"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="A110:D110"/>
-    <mergeCell ref="A111:D111"/>
-    <mergeCell ref="A112:D112"/>
-    <mergeCell ref="A118:D118"/>
-    <mergeCell ref="A119:D119"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="A68:D68"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A70:D70"/>
-    <mergeCell ref="A85:D85"/>
-    <mergeCell ref="A86:D86"/>
-    <mergeCell ref="A87:D87"/>
-  </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>